<commit_message>
Add ASIC and glass fiber theme seeds
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -3977,17 +3977,25 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>非主流</t>
+          <t>主流</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>塑膠工業</t>
-        </is>
-      </c>
-      <c r="F188" t="inlineStr"/>
+          <t>玻纖布</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>PCB_CCL_ABF材料</t>
+        </is>
+      </c>
       <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>user_authorized_seed_20260530</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7844,10 +7852,14 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
+          <t>玻纖布</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
           <t>PCB_CCL_ABF材料</t>
         </is>
       </c>
-      <c r="F369" t="inlineStr"/>
       <c r="G369" t="inlineStr"/>
       <c r="H369" t="inlineStr">
         <is>
@@ -8010,10 +8022,14 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
+          <t>玻纖布</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
           <t>PCB_CCL_ABF材料</t>
         </is>
       </c>
-      <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr"/>
       <c r="H376" t="inlineStr">
         <is>
@@ -28529,11 +28545,27 @@
         </is>
       </c>
       <c r="C317" t="inlineStr"/>
-      <c r="D317" t="inlineStr"/>
-      <c r="E317" t="inlineStr"/>
-      <c r="F317" t="inlineStr"/>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>主流</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>玻纖布</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>PCB_CCL_ABF材料</t>
+        </is>
+      </c>
       <c r="G317" t="inlineStr"/>
-      <c r="H317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>user_authorized_seed_20260530</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -29317,11 +29349,27 @@
         </is>
       </c>
       <c r="C353" t="inlineStr"/>
-      <c r="D353" t="inlineStr"/>
-      <c r="E353" t="inlineStr"/>
-      <c r="F353" t="inlineStr"/>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>主流</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>玻纖布</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>PCB_CCL_ABF材料</t>
+        </is>
+      </c>
       <c r="G353" t="inlineStr"/>
-      <c r="H353" t="inlineStr"/>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>user_authorized_seed_20260530</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -35045,15 +35093,23 @@
           <t>半導體業</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>主流</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>半導體業</t>
+          <t>矽智財_ASIC</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>user_authorized_seed_20260530</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">

</xml_diff>

<commit_message>
Add specialty material theme override
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -7295,19 +7295,27 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>非主流</t>
+          <t>主流</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>化學工業</t>
-        </is>
-      </c>
-      <c r="F335" t="inlineStr"/>
-      <c r="G335" t="inlineStr"/>
+          <t>特化材料</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>特化化學</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>電子材料</t>
+        </is>
+      </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>provisional_industry_mapping</t>
+          <t>user_authorized_specialty_theme_20260530</t>
         </is>
       </c>
     </row>
@@ -7497,11 +7505,31 @@
         </is>
       </c>
       <c r="C343" t="inlineStr"/>
-      <c r="D343" t="inlineStr"/>
-      <c r="E343" t="inlineStr"/>
-      <c r="F343" t="inlineStr"/>
-      <c r="G343" t="inlineStr"/>
-      <c r="H343" t="inlineStr"/>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>主流</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>特化材料</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>特化化學</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>電子材料</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>user_authorized_specialty_theme_20260530</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">

</xml_diff>

<commit_message>
Stabilize daily candidate data pipeline audit
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -460,46 +460,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>族群1</t>
+          <t>基本族群</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>填最重要族群，例如機器人自動化、玻纖布、低軌衛星、被動元件。</t>
+          <t>每檔股票都應有一個常態分類，例如電機機械、通信網路、塑膠、金融保險。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>族群2/族群3/族群4/族群5</t>
+          <t>熱門族群1～熱門族群5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>同一股票有多個族群時再填。</t>
+          <t>只填資金題材或你要納入熱門族群模型的標籤，例如機器人自動化、玻纖布、低軌衛星、被動元件。留空時不進入熱門族群回檔模型。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>產業預設/題材預設/最終分流/雙重身分</t>
+          <t>備註</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
-        <is>
-          <t>程式參考欄，通常不用改。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>備註</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
         <is>
           <t>需要說明來源或例外時填。</t>
         </is>
@@ -516,26 +504,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,70 +538,40 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>基本族群</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>族群1</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>族群2</t>
+          <t>熱門族群1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>族群3</t>
+          <t>熱門族群2</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>族群4</t>
+          <t>熱門族群3</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>族群5</t>
+          <t>熱門族群4</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>產業預設</t>
+          <t>熱門族群5</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>題材預設</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>最終分流</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>雙重身分</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>report_line_memberships</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>mainstream_report_eligible</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>non_mainstream_report_eligible</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -643,50 +595,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>電機機械</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>主流</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>機器人自動化</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>主流</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>主流</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>主流</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>mainstream</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh stock theme taxonomy outputs
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,12 +438,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>欄位</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>填寫方式</t>
         </is>
@@ -513,57 +525,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -18625,57 +18637,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -37373,57 +37385,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -55945,57 +55957,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -73809,57 +73821,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>

</xml_diff>

<commit_message>
Refine bottom volume attack model and daily outputs
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,12 +438,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>欄位</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>填寫方式</t>
         </is>
@@ -513,57 +525,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -18621,57 +18633,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -37369,57 +37381,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -55941,57 +55953,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -73809,57 +73821,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>

</xml_diff>

<commit_message>
[codex] Guard daily freshness publish and restore 20260611 sources (#36)
* Guard daily freshness publish and restore 20260611 sources

* Preserve same-date warrant data on fetch fallback

* Update daily report artifacts and packets

* Publish daily report readme and ChatGPT entries

---------

Co-authored-by: Codex <codex@local>
Co-authored-by: github-actions <github-actions@github.com>
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -17871,12 +17871,12 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E483" t="inlineStr">
@@ -23666,12 +23666,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>其他業</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -85865,12 +85865,12 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -86479,12 +86479,12 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -86681,12 +86681,12 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">

</xml_diff>

<commit_message>
Resolve daily group rotation theme display
</commit_message>
<xml_diff>
--- a/docs/latest/stock_theme_manual_fill_template_latest.xlsx
+++ b/docs/latest/stock_theme_manual_fill_template_latest.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,12 +438,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>欄位</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>填寫方式</t>
         </is>
@@ -513,57 +525,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -582,12 +594,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -615,12 +627,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -648,12 +660,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -681,12 +693,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -714,12 +726,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -747,12 +759,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -780,12 +792,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -813,12 +825,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -846,12 +858,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -879,12 +891,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -912,12 +924,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -945,12 +957,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -978,12 +990,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1011,12 +1023,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1044,12 +1056,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1077,12 +1089,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1110,12 +1122,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1143,12 +1155,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1176,12 +1188,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1209,12 +1221,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1242,12 +1254,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1275,12 +1287,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1308,12 +1320,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1341,12 +1353,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1374,12 +1386,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1407,12 +1419,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1440,12 +1452,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1473,12 +1485,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1506,12 +1518,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1539,12 +1551,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1572,12 +1584,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1605,12 +1617,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1638,12 +1650,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1671,12 +1683,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1704,12 +1716,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1737,12 +1749,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1770,12 +1782,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1803,12 +1815,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1836,12 +1848,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1869,12 +1881,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1902,12 +1914,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1935,12 +1947,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1968,12 +1980,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2001,12 +2013,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2034,12 +2046,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2067,12 +2079,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2100,12 +2112,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2133,12 +2145,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2166,12 +2178,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2199,12 +2211,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2232,12 +2244,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2265,12 +2277,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2298,12 +2310,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2331,12 +2343,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2364,12 +2376,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2397,12 +2409,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2430,12 +2442,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2463,12 +2475,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2496,12 +2508,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2529,12 +2541,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2562,12 +2574,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2595,12 +2607,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2628,12 +2640,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2661,12 +2673,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2694,12 +2706,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2727,12 +2739,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2760,12 +2772,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2793,12 +2805,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2826,12 +2838,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2859,12 +2871,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2892,12 +2904,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2925,12 +2937,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2958,12 +2970,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2991,12 +3003,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3024,12 +3036,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3057,12 +3069,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3090,12 +3102,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3123,12 +3135,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3156,12 +3168,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3189,12 +3201,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3222,12 +3234,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3255,12 +3267,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3288,12 +3300,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3321,12 +3333,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3354,12 +3366,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3387,12 +3399,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3420,12 +3432,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3453,12 +3465,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3486,12 +3498,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3519,12 +3531,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -3552,12 +3564,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -3585,12 +3597,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -3618,12 +3630,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -3651,12 +3663,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -3684,12 +3696,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -3717,12 +3729,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -3750,12 +3762,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3783,12 +3795,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -3816,12 +3828,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -3849,12 +3861,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -3882,12 +3894,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -3915,12 +3927,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -3948,12 +3960,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3981,12 +3993,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4014,12 +4026,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4047,12 +4059,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4080,12 +4092,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -4113,12 +4125,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4146,12 +4158,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4179,12 +4191,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4212,12 +4224,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4245,12 +4257,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -4278,12 +4290,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4311,12 +4323,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -4344,12 +4356,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -4377,12 +4389,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -4410,12 +4422,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4443,12 +4455,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -4476,12 +4488,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -4509,12 +4521,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -4542,12 +4554,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -4575,12 +4587,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -4608,12 +4620,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -4641,12 +4653,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -4674,12 +4686,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -4707,12 +4719,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -4740,12 +4752,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -4773,12 +4785,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -4806,12 +4818,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -4839,12 +4851,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -4872,12 +4884,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -4905,12 +4917,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -4938,12 +4950,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -4971,12 +4983,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5004,12 +5016,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -5037,12 +5049,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -5070,12 +5082,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -5103,12 +5115,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -5136,12 +5148,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -5169,12 +5181,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -5202,12 +5214,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -5235,12 +5247,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -5268,12 +5280,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -5301,12 +5313,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -5334,12 +5346,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -5367,12 +5379,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -5400,12 +5412,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -5433,12 +5445,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -5466,12 +5478,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -5499,12 +5511,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -5532,12 +5544,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -5565,12 +5577,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -5598,12 +5610,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>指數/ETF/ETN商品</t>
+          <t>指數 / ETF / ETN商品</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -7781,12 +7793,12 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>TPU材料 / 工業複合材料</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>TPU材料 / 工業複合材料</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -17871,12 +17883,12 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>房地產代銷 / 建設服務</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>房地產代銷 / 建設服務</t>
         </is>
       </c>
       <c r="E483" t="inlineStr">
@@ -18621,57 +18633,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -37361,57 +37373,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -52123,12 +52135,12 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>租賃金融 / 企業融資</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>租賃金融 / 企業融資</t>
         </is>
       </c>
       <c r="E399" t="inlineStr">
@@ -55933,57 +55945,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -61728,12 +61740,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>TPU材料 / 工業複合材料</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>TPU材料 / 工業複合材料</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -67116,12 +67128,12 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>投資控股 / 創投</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>投資控股 / 創投</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -73805,57 +73817,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>股票代號</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>股票名稱</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>上市櫃產業</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>基本族群</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>主流/非主流</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>熱門族群1</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>熱門族群2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>熱門族群3</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>熱門族群4</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>熱門族群5</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -78427,12 +78439,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>權證/衍生商品</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>其他業</t>
+          <t>權證/衍生商品</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -85326,12 +85338,12 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -85363,12 +85375,12 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -85400,12 +85412,12 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -85437,12 +85449,12 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -85474,12 +85486,12 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -85511,12 +85523,12 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -85548,12 +85560,12 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -85585,12 +85597,12 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -85622,12 +85634,12 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -85659,12 +85671,12 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>DR / 外國上市</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -85865,12 +85877,12 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>包材 / 容器製造</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>包材 / 容器製造</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -86071,12 +86083,12 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>保全 / 智慧安防服務</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>保全 / 智慧安防服務</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -86479,12 +86491,12 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工程承攬 / EPC服務</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>工程承攬 / EPC服務</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -86714,12 +86726,12 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>汽車金融 / 分期租賃</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>汽車金融 / 分期租賃</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -86850,12 +86862,12 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>建設營造 / 商用不動產</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>建設營造 / 商用不動產</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">

</xml_diff>